<commit_message>
Gộp run_a + run_b, báo cáo run 0-9
</commit_message>
<xml_diff>
--- a/results/bang_tong_hop_luan_van.xlsx
+++ b/results/bang_tong_hop_luan_van.xlsx
@@ -494,21 +494,21 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.022 ± 0.037</t>
+          <t>4.019 ± 0.031</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[3.976, 4.068]</t>
+          <t>[3.997, 4.041]</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>38.143 ± 0.211</t>
+          <t>38.120 ± 0.183</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,12 +518,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.919</t>
+          <t>3.916</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>14.71</t>
+          <t>29.25</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -544,36 +544,36 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>15.009 ± 0.305</t>
+          <t>15.073 ± 0.282</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[14.631, 15.388]</t>
+          <t>[14.871, 15.275]</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>64.327 ± 1.350</t>
+          <t>64.492 ± 1.037</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.1225</t>
+          <t>0.1228</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>14.906</t>
+          <t>14.971</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5.17</t>
+          <t>5.04</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -590,21 +590,21 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.511 ± 0.031</t>
+          <t>5.509 ± 0.032</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[5.472, 5.550]</t>
+          <t>[5.486, 5.532]</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>43.509 ± 0.130</t>
+          <t>43.449 ± 0.157</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -614,12 +614,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>5.409</t>
+          <t>5.408</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -636,21 +636,21 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.738 ± 0.036</t>
+          <t>4.734 ± 0.025</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[4.693, 4.783]</t>
+          <t>[4.716, 4.752]</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>40.129 ± 0.176</t>
+          <t>40.108 ± 0.126</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4.634</t>
+          <t>4.631</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.60</t>
+          <t>21.13</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -682,32 +682,32 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.543 ± 0.796</t>
+          <t>5.780 ± 0.836</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[4.554, 6.531]</t>
+          <t>[5.182, 6.377]</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>39.134 ± 0.732</t>
+          <t>39.524 ± 1.162</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.0743</t>
+          <t>0.0758</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>6.59</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -724,32 +724,32 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8.437 ± 0.022</t>
+          <t>8.425 ± 0.024</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[8.410, 8.465]</t>
+          <t>[8.408, 8.442]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>55.752 ± 0.066</t>
+          <t>55.739 ± 0.056</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.0919</t>
+          <t>0.0918</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -766,21 +766,21 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.723 ± 0.004</t>
+          <t>0.723 ± 0.003</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[0.718, 0.728]</t>
+          <t>[0.721, 0.726]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>5.452 ± 0.024</t>
+          <t>5.450 ± 0.017</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>10.83</t>
+          <t>12.27</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -816,21 +816,21 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.736 ± 0.005</t>
+          <t>0.737 ± 0.004</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[0.729, 0.743]</t>
+          <t>[0.734, 0.740]</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>5.402 ± 0.010</t>
+          <t>5.398 ± 0.008</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -840,12 +840,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.469</t>
+          <t>0.468</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>4.47</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -862,26 +862,26 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.914 ± 0.003</t>
+          <t>0.915 ± 0.003</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>[0.910, 0.918]</t>
+          <t>[0.913, 0.918]</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>5.858 ± 0.011</t>
+          <t>5.865 ± 0.015</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.0302</t>
+          <t>0.0303</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -908,21 +908,21 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.752 ± 0.001</t>
+          <t>0.751 ± 0.001</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[0.751, 0.753]</t>
+          <t>[0.751, 0.752]</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5.755 ± 0.006</t>
+          <t>5.758 ± 0.005</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>6.03</t>
+          <t>6.64</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -954,21 +954,21 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.919 ± 0.003</t>
+          <t>0.920 ± 0.003</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>[0.915, 0.924]</t>
+          <t>[0.918, 0.922]</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6.004 ± 0.025</t>
+          <t>6.006 ± 0.023</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -979,7 +979,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>7.81</t>
+          <t>8.38</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -996,21 +996,21 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.914 ± 0.001</t>
+          <t>0.915 ± 0.003</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[0.913, 0.915]</t>
+          <t>[0.912, 0.917]</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>5.907 ± 0.012</t>
+          <t>5.902 ± 0.019</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1021,7 +1021,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1038,36 +1038,36 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.846 ± 0.007</t>
+          <t>1.844 ± 0.007</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>[1.838, 1.855]</t>
+          <t>[1.839, 1.849]</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>16.285 ± 0.008</t>
+          <t>16.273 ± 0.017</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.0430</t>
+          <t>0.0429</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1.318</t>
+          <t>1.317</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>14.00</t>
+          <t>11.18</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1088,36 +1088,36 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.966 ± 0.016</t>
+          <t>1.972 ± 0.014</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[1.946, 1.985]</t>
+          <t>[1.962, 1.982]</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>16.924 ± 0.021</t>
+          <t>16.933 ± 0.022</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.0443</t>
+          <t>0.0444</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.454</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.67</t>
+          <t>4.48</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1134,21 +1134,21 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.764 ± 0.013</t>
+          <t>2.764 ± 0.014</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>[2.748, 2.780]</t>
+          <t>[2.754, 2.773]</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>17.461 ± 0.021</t>
+          <t>17.470 ± 0.022</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1158,12 +1158,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1.122</t>
+          <t>1.123</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1180,21 +1180,21 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.858 ± 0.006</t>
+          <t>1.855 ± 0.006</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>[1.851, 1.865]</t>
+          <t>[1.851, 1.859]</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>16.283 ± 0.010</t>
+          <t>16.271 ± 0.017</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1.336</t>
+          <t>1.334</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>6.72</t>
+          <t>4.42</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1226,21 +1226,21 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.926 ± 0.040</t>
+          <t>2.922 ± 0.036</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>[2.876, 2.976]</t>
+          <t>[2.896, 2.948]</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>17.656 ± 0.049</t>
+          <t>17.654 ± 0.045</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1251,7 +1251,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.99</t>
+          <t>4.45</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1268,32 +1268,32 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.709 ± 0.039</t>
+          <t>2.720 ± 0.035</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>[2.661, 2.758]</t>
+          <t>[2.696, 2.745]</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>17.476 ± 0.063</t>
+          <t>17.493 ± 0.058</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0.0520</t>
+          <t>0.0522</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1366,23 +1366,23 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>-10.98723905893166</v>
+        <v>-11.05460649621575</v>
       </c>
       <c r="E2" t="n">
-        <v>-85.8916419254025</v>
+        <v>-132.4115239320759</v>
       </c>
       <c r="F2" t="n">
-        <v>1.101425879156631e-07</v>
+        <v>4.06094405281102e-16</v>
       </c>
       <c r="G2" t="n">
-        <v>-130.5624297605268</v>
+        <v>-133.2526074656401</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -1398,23 +1398,23 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.48872469817672</v>
+        <v>-1.4904476375717</v>
       </c>
       <c r="E3" t="n">
-        <v>-171.6069487166656</v>
+        <v>-150.1685036724641</v>
       </c>
       <c r="F3" t="n">
-        <v>6.916931322219701e-09</v>
+        <v>1.30903790109229e-16</v>
       </c>
       <c r="G3" t="n">
-        <v>-62.15399422614647</v>
+        <v>-64.960572658375</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -1430,23 +1430,23 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.7161995533130801</v>
+        <v>-0.7150730389999599</v>
       </c>
       <c r="E4" t="n">
-        <v>-74.86750974466149</v>
+        <v>-101.1338532680911</v>
       </c>
       <c r="F4" t="n">
-        <v>1.907485885208829e-07</v>
+        <v>4.583942681855937e-15</v>
       </c>
       <c r="G4" t="n">
-        <v>-72.88717346681429</v>
+        <v>-73.45343126157982</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -1462,16 +1462,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>-1.520838175462</v>
+        <v>-1.76089641013437</v>
       </c>
       <c r="E5" t="n">
-        <v>-4.282291996974505</v>
+        <v>-6.609282374909742</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01282430538553298</v>
+        <v>9.822108816958828e-05</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -1488,16 +1488,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>-4.415407347199561</v>
+        <v>-4.406419965737021</v>
       </c>
       <c r="E6" t="n">
-        <v>-368.4273245843883</v>
+        <v>-568.6317076719375</v>
       </c>
       <c r="F6" t="n">
-        <v>3.256286369182417e-10</v>
+        <v>8.191090494751265e-22</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -1514,23 +1514,23 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.01326038596432002</v>
+        <v>-0.01373765948309001</v>
       </c>
       <c r="E7" t="n">
-        <v>-11.44297856437088</v>
+        <v>-17.35746294670894</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0003328134840953929</v>
+        <v>3.156370749718454e-08</v>
       </c>
       <c r="G7" t="n">
-        <v>-1.519744462916579</v>
+        <v>-1.733311316646641</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>2/10</t>
         </is>
       </c>
     </row>
@@ -1546,23 +1546,23 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.19143416329186</v>
+        <v>-0.19222215306585</v>
       </c>
       <c r="E8" t="n">
-        <v>-80.62852309367295</v>
+        <v>-155.7384523866793</v>
       </c>
       <c r="F8" t="n">
-        <v>1.418244794503242e-07</v>
+        <v>9.432981928465741e-17</v>
       </c>
       <c r="G8" t="n">
-        <v>-1.355340247890647</v>
+        <v>-1.356025575165335</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>0/10</t>
         </is>
       </c>
     </row>
@@ -1578,23 +1578,23 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.02876000697514003</v>
+        <v>-0.02829452837595001</v>
       </c>
       <c r="E9" t="n">
-        <v>-14.01651623573573</v>
+        <v>-23.75546683908001</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0001503126983597008</v>
+        <v>1.980999668464163e-09</v>
       </c>
       <c r="G9" t="n">
-        <v>-1.402625426066681</v>
+        <v>-1.386066351074393</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0/5</t>
+          <t>0/10</t>
         </is>
       </c>
     </row>
@@ -1610,16 +1610,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.19636919487766</v>
+        <v>-0.19690741809636</v>
       </c>
       <c r="E10" t="n">
-        <v>-79.97172690243985</v>
+        <v>-156.0556259777293</v>
       </c>
       <c r="F10" t="n">
-        <v>1.465388500204142e-07</v>
+        <v>9.261887467282744e-17</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -1636,16 +1636,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.19112236190578</v>
+        <v>-0.19155532057637</v>
       </c>
       <c r="E11" t="n">
-        <v>-102.4525499707147</v>
+        <v>-110.1569652444044</v>
       </c>
       <c r="F11" t="n">
-        <v>5.442323813061019e-08</v>
+        <v>2.125425703309742e-15</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -1662,23 +1662,23 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.1193333966132401</v>
+        <v>-0.12782484623257</v>
       </c>
       <c r="E12" t="n">
-        <v>-17.838194593865</v>
+        <v>-26.04539837495844</v>
       </c>
       <c r="F12" t="n">
-        <v>5.803674838326021e-05</v>
+        <v>8.747284717891702e-10</v>
       </c>
       <c r="G12" t="n">
-        <v>-7.419937626466552</v>
+        <v>-8.44622378922932</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -1694,23 +1694,23 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.9174971116687801</v>
+        <v>-0.91941098982443</v>
       </c>
       <c r="E13" t="n">
-        <v>-151.6399007891579</v>
+        <v>-226.5773350136269</v>
       </c>
       <c r="F13" t="n">
-        <v>1.134413491017134e-08</v>
+        <v>3.233040990248141e-18</v>
       </c>
       <c r="G13" t="n">
-        <v>-3.320254982365578</v>
+        <v>-3.348014668629843</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -1726,23 +1726,23 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.01164480817576002</v>
+        <v>-0.01125009055259999</v>
       </c>
       <c r="E14" t="n">
-        <v>-4.313765838419512</v>
+        <v>-6.326488588186361</v>
       </c>
       <c r="F14" t="n">
-        <v>0.01250878691719327</v>
+        <v>0.0001366233149015208</v>
       </c>
       <c r="G14" t="n">
-        <v>-5.250184722229029</v>
+        <v>-5.228054420323346</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>10/10</t>
         </is>
       </c>
     </row>
@@ -1758,16 +1758,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>-1.07993815324208</v>
+        <v>-1.07772971377161</v>
       </c>
       <c r="E15" t="n">
-        <v>-58.26223774440352</v>
+        <v>-95.00592901410755</v>
       </c>
       <c r="F15" t="n">
-        <v>5.196969247050447e-07</v>
+        <v>8.041624748140805e-15</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -1784,16 +1784,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.86303679831854</v>
+        <v>-0.8761000028426998</v>
       </c>
       <c r="E16" t="n">
-        <v>-43.59573311052795</v>
+        <v>-69.3988378502733</v>
       </c>
       <c r="F16" t="n">
-        <v>1.655211422962183e-06</v>
+        <v>1.353268814338055e-13</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -1866,19 +1866,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>1.857905377814689</v>
+        <v>1.85542242525322</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0057493477800946</v>
+        <v>0.0056758332248065</v>
       </c>
       <c r="F2" t="n">
-        <v>16.28336155695142</v>
+        <v>16.27128923866768</v>
       </c>
       <c r="G2" t="n">
-        <v>1.335649844259024</v>
+        <v>1.33415566524484</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>1.860145608988091</v>
+        <v>1.856512639876631</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0126660967715038</v>
+        <v>0.0117248828481232</v>
       </c>
       <c r="F3" t="n">
-        <v>16.45452594510792</v>
+        <v>16.44401252117571</v>
       </c>
       <c r="G3" t="n">
-        <v>1.20576499029994</v>
+        <v>1.20654879137869</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1930,19 +1930,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>1.84626056911088</v>
+        <v>1.844172334721</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0069551461965144</v>
+        <v>0.0070639954995347</v>
       </c>
       <c r="F4" t="n">
-        <v>16.28494922642858</v>
+        <v>16.27308528075617</v>
       </c>
       <c r="G4" t="n">
-        <v>1.318189571611583</v>
+        <v>1.31729175336654</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>1.84626056911088</v>
+        <v>1.844172334721</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0069551461965144</v>
+        <v>0.0070639954995347</v>
       </c>
       <c r="F5" t="n">
-        <v>16.28494922642858</v>
+        <v>16.27308528075617</v>
       </c>
       <c r="G5" t="n">
-        <v>1.318189571611583</v>
+        <v>1.31729175336654</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1994,19 +1994,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>2.644744431958617</v>
+        <v>2.64113288497675</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0068190091108787</v>
+        <v>0.009848090501068</v>
       </c>
       <c r="F6" t="n">
-        <v>17.35025351246182</v>
+        <v>17.35646219493476</v>
       </c>
       <c r="G6" t="n">
-        <v>1.118461997248232</v>
+        <v>1.11947560217227</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -2026,19 +2026,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
-        <v>1.844778053743166</v>
+        <v>1.84262493317787</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0069237622286674</v>
+        <v>0.0067377836505502</v>
       </c>
       <c r="F7" t="n">
-        <v>16.28855873985068</v>
+        <v>16.27679099472646</v>
       </c>
       <c r="G7" t="n">
-        <v>1.315243169665337</v>
+        <v>1.31426325533534</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -2058,19 +2058,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D8" t="n">
-        <v>1.85692007923777</v>
+        <v>1.85449727086676</v>
       </c>
       <c r="E8" t="n">
-        <v>0.00577171458981</v>
+        <v>0.0056031317590589</v>
       </c>
       <c r="F8" t="n">
-        <v>16.27934929452714</v>
+        <v>16.26733716222089</v>
       </c>
       <c r="G8" t="n">
-        <v>1.334813446737826</v>
+        <v>1.33338901214297</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -2090,19 +2090,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D9" t="n">
-        <v>1.846236271433647</v>
+        <v>1.84415014027524</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0069673424965228</v>
+        <v>0.0070770894663327</v>
       </c>
       <c r="F9" t="n">
-        <v>16.28488227085518</v>
+        <v>16.27302334255481</v>
       </c>
       <c r="G9" t="n">
-        <v>1.318172365427017</v>
+        <v>1.31727587431666</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -2122,19 +2122,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>1.864544118345822</v>
+        <v>1.86547583273741</v>
       </c>
       <c r="E10" t="n">
-        <v>0.008749365382702001</v>
+        <v>0.0066293185320843</v>
       </c>
       <c r="F10" t="n">
-        <v>16.47510965299272</v>
+        <v>16.478486379425</v>
       </c>
       <c r="G10" t="n">
-        <v>1.194104901514947</v>
+        <v>1.19666728423904</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -2154,19 +2154,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>0.91427570363193</v>
+        <v>0.9153410589277799</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0031850526344003</v>
+        <v>0.0033116687248463</v>
       </c>
       <c r="F11" t="n">
-        <v>5.85759029773599</v>
+        <v>5.86496127502438</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4545478615909815</v>
+        <v>0.45514557568818</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -2186,19 +2186,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8510287756237741</v>
+        <v>0.85232361120235</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0061829091746289</v>
+        <v>0.0048440398945429</v>
       </c>
       <c r="F12" t="n">
-        <v>5.510256756280518</v>
+        <v>5.50946628915696</v>
       </c>
       <c r="G12" t="n">
-        <v>0.4450094071216881</v>
+        <v>0.4451932560186299</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -2218,19 +2218,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>0.722841540340072</v>
+        <v>0.7231189058619301</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0040630505169623</v>
+        <v>0.0033546768691779</v>
       </c>
       <c r="F13" t="n">
-        <v>5.452237248361236</v>
+        <v>5.44958988666686</v>
       </c>
       <c r="G13" t="n">
-        <v>0.4461191885638982</v>
+        <v>0.4460960539290299</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -2250,19 +2250,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D14" t="n">
-        <v>0.722841540340072</v>
+        <v>0.7231189058619301</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0040630505169623</v>
+        <v>0.0033546768691779</v>
       </c>
       <c r="F14" t="n">
-        <v>5.452237248361236</v>
+        <v>5.44958988666686</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4461191885638982</v>
+        <v>0.4460960539290299</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -2282,19 +2282,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>0.7582785689870656</v>
+        <v>0.75856117987265</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0052093039463359</v>
+        <v>0.0038458346062419</v>
       </c>
       <c r="F15" t="n">
-        <v>5.430623260111981</v>
+        <v>5.42821716656532</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4481257987208664</v>
+        <v>0.44827491219616</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -2314,19 +2314,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7266923395433541</v>
+        <v>0.7262794769863101</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0014705966712758</v>
+        <v>0.0021182788516633</v>
       </c>
       <c r="F16" t="n">
-        <v>5.732247976816517</v>
+        <v>5.735604039446379</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4448495979886502</v>
+        <v>0.4450516134965699</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -2346,19 +2346,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>0.7223726835518653</v>
+        <v>0.72191176017849</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0008640163599357</v>
+        <v>0.0008781350014297</v>
       </c>
       <c r="F17" t="n">
-        <v>5.438262470795229</v>
+        <v>5.43711454454313</v>
       </c>
       <c r="G17" t="n">
-        <v>0.4558354383334517</v>
+        <v>0.45524353336073</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2378,19 +2378,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7410755516798756</v>
+        <v>0.74091611670415</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0032180411045608</v>
+        <v>0.0037631107973505</v>
       </c>
       <c r="F18" t="n">
-        <v>5.453585297250554</v>
+        <v>5.45100807217483</v>
       </c>
       <c r="G18" t="n">
-        <v>0.4451437620446086</v>
+        <v>0.44516582274806</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2410,19 +2410,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D19" t="n">
-        <v>0.7225165098206724</v>
+        <v>0.723092018425</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0027066772685963</v>
+        <v>0.0020265280174013</v>
       </c>
       <c r="F19" t="n">
-        <v>5.508844561549465</v>
+        <v>5.511232381043399</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4443507816176861</v>
+        <v>0.4441896278876299</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2442,19 +2442,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D20" t="n">
-        <v>4.738176530001774</v>
+        <v>4.73377582463069</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0363812894204518</v>
+        <v>0.0253211470927584</v>
       </c>
       <c r="F20" t="n">
-        <v>40.12912620820403</v>
+        <v>40.10800676246193</v>
       </c>
       <c r="G20" t="n">
-        <v>4.634472634643316</v>
+        <v>4.630854586139261</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2474,19 +2474,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D21" t="n">
-        <v>4.701268618182302</v>
+        <v>4.69638969758302</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0355753223068005</v>
+        <v>0.0255099526314482</v>
       </c>
       <c r="F21" t="n">
-        <v>39.90089117656464</v>
+        <v>39.86725146728902</v>
       </c>
       <c r="G21" t="n">
-        <v>4.598081205040216</v>
+        <v>4.59389346651728</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2506,19 +2506,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>4.021976973990603</v>
+        <v>4.01870278376248</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0369914240265272</v>
+        <v>0.0308644896186037</v>
       </c>
       <c r="F22" t="n">
-        <v>38.14258726204638</v>
+        <v>38.12020762370782</v>
       </c>
       <c r="G22" t="n">
-        <v>3.918661735951901</v>
+        <v>3.91609822399909</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2538,19 +2538,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>4.696577115174799</v>
+        <v>4.691766102669431</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0356865911548164</v>
+        <v>0.0255429959797806</v>
       </c>
       <c r="F23" t="n">
-        <v>39.87277015049689</v>
+        <v>39.83655400606948</v>
       </c>
       <c r="G23" t="n">
-        <v>4.593465570360422</v>
+        <v>4.58932742476456</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -2570,19 +2570,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>4.855046349028758</v>
+        <v>4.84587116290118</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0352274810722637</v>
+        <v>0.0396123974618711</v>
       </c>
       <c r="F24" t="n">
-        <v>42.01459466677987</v>
+        <v>41.95831250686768</v>
       </c>
       <c r="G24" t="n">
-        <v>4.75364476442337</v>
+        <v>4.744610190391489</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2602,19 +2602,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D25" t="n">
-        <v>4.693979906296111</v>
+        <v>4.6891438774474</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0356357111968634</v>
+        <v>0.0255231801735128</v>
       </c>
       <c r="F25" t="n">
-        <v>39.85685364178052</v>
+        <v>39.82020015131911</v>
       </c>
       <c r="G25" t="n">
-        <v>4.590860195457935</v>
+        <v>4.586695041507429</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2634,19 +2634,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D26" t="n">
-        <v>4.156832958401374</v>
+        <v>4.15575156622608</v>
       </c>
       <c r="E26" t="n">
-        <v>0.0425580242111096</v>
+        <v>0.0318561129892728</v>
       </c>
       <c r="F26" t="n">
-        <v>38.78982504716802</v>
+        <v>38.78727794676083</v>
       </c>
       <c r="G26" t="n">
-        <v>4.053048975765705</v>
+        <v>4.05275369994338</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2666,19 +2666,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D27" t="n">
-        <v>4.021976973990603</v>
+        <v>4.01870278376248</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0369914240265272</v>
+        <v>0.0308644896186037</v>
       </c>
       <c r="F27" t="n">
-        <v>38.14258726204638</v>
+        <v>38.12020762370782</v>
       </c>
       <c r="G27" t="n">
-        <v>3.918661735951901</v>
+        <v>3.91609822399909</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -2698,19 +2698,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D28" t="n">
-        <v>6.322681945602771</v>
+        <v>6.32965748029872</v>
       </c>
       <c r="E28" t="n">
-        <v>0.065276147932118</v>
+        <v>0.0502401345630376</v>
       </c>
       <c r="F28" t="n">
-        <v>46.26426224880567</v>
+        <v>46.30817633208967</v>
       </c>
       <c r="G28" t="n">
-        <v>6.221825536340475</v>
+        <v>6.22953511774535</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>

</xml_diff>